<commit_message>
fix(cirrus): share equilibration tables
</commit_message>
<xml_diff>
--- a/test_data/examples/smeaheia/smeaheia_workbook.xlsx
+++ b/test_data/examples/smeaheia/smeaheia_workbook.xlsx
@@ -1545,16 +1545,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1500</v>
+        <v>1282.5</v>
       </c>
       <c r="E2" t="n">
-        <v>150</v>
+        <v>129.99</v>
       </c>
       <c r="F2" t="n">
-        <v>1550</v>
+        <v>1282.5</v>
       </c>
       <c r="G2" t="n">
-        <v>155</v>
+        <v>129.99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>